<commit_message>
loads of changes sheesh
</commit_message>
<xml_diff>
--- a/HMRC Info.xlsx
+++ b/HMRC Info.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\WCale\Desktop\flonancial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A3AA4633-03E0-4B59-A370-1B0883EE195A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E28FCCDC-1C1F-4AF8-B2C5-BA89690B16B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28230" yWindow="-570" windowWidth="21600" windowHeight="14700" xr2:uid="{FBE2A083-299E-45AF-96C3-B1141BD30B63}"/>
+    <workbookView xWindow="-28920" yWindow="-1260" windowWidth="29040" windowHeight="15720" xr2:uid="{FBE2A083-299E-45AF-96C3-B1141BD30B63}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,6 +33,35 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+  <si>
+    <t>At a minimum, digital records must include the date, amount, and category of each transaction — income received (sales, rental payments, other receipts) and allowable expenses (supplies, travel, professional fees, repairs). Making Tax Digital</t>
+  </si>
+  <si>
+    <t>And crucially for your target market — relevant persons under the VAT threshold may choose to categorise their digital records of income and expenses in less detail. Ross Martin</t>
+  </si>
+  <si>
+    <t>The VAT threshold is £90,000. Your target users — simple sole traders and landlords — are almost certainly under that. So they qualify for simplified categorisation.</t>
+  </si>
+  <si>
+    <t>So here's the minimum compliant data model for Flonancial:</t>
+  </si>
+  <si>
+    <t>Each transaction record needs just three fields:</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>Type — income or expense (that's it for under-£90k users, no detailed categories needed)</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -66,8 +95,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -402,9 +434,53 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77D67572-3417-4A0C-BE24-135E508CB379}">
-  <dimension ref="A1"/>
+  <dimension ref="B2:B10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
+  <cols>
+    <col min="2" max="2" width="93.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:2" ht="51.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="2:2" x14ac:dyDescent="0.35">
+      <c r="B10" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>